<commit_message>
refactor(Proveedores - Orden de compra Excel): Agregados datos al reporte
</commit_message>
<xml_diff>
--- a/application/views/reportes/plantillas/proveedores_orden_compra.xlsx
+++ b/application/views/reportes/plantillas/proveedores_orden_compra.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\proyectos\simon-bolivar\application\views\reportes\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB556FA7-3994-433C-8901-D43915A2BF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE21E3B1-57D9-4B97-BBE7-B20EC2C1C04E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{AB0910D4-337B-4AA8-B272-A0A042017033}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>CENTRO DE OPERACIÓN</t>
   </si>
@@ -97,7 +97,7 @@
     <t>PROVEEDOR ÚLTIMA COMPRA</t>
   </si>
   <si>
-    <t>Tipo docto</t>
+    <t>PROVEEDOR SEGUNDA COTIZACIÓN</t>
   </si>
 </sst>
 </file>
@@ -594,7 +594,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3254C59D-5EEE-4ABA-B049-38AD83484C92}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -609,15 +609,15 @@
     <col min="10" max="10" width="13.28515625" customWidth="1"/>
     <col min="11" max="11" width="22" customWidth="1"/>
     <col min="15" max="15" width="23" customWidth="1"/>
-    <col min="16" max="16" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="27.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -656,6 +656,9 @@
       </c>
       <c r="P1" s="1" t="s">
         <v>18</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>